<commit_message>
Re-cut the Nov 9 CSS retest targets off the 400 and 200
Two sessions say the Sep 21 400 was not a maximal effort: the Oct 5 warm-up 400 came in at 7:07.5, within 1.5s of the all-out test, and the 5x200 that followed held 1:47.6/100 without fading. The old target table chased a CSS number off that soft baseline, which measures the gap between the two swims rather than either swim. Retarget the 400 and 200 directly, add a floor row so an honest test that gains nothing is still legible as a result, and note the easy warm-up requirement.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Abid — Fall 2026 Training Block.xlsx
+++ b/Abid — Fall 2026 Training Block.xlsx
@@ -12385,7 +12385,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -12471,7 +12471,7 @@
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>First CSS test. The 400/200 ratio is 2.13, inside the normal 2.10–2.20 band, so the number is internally consistent and the speed-to-endurance balance is healthy.</t>
+          <t>First CSS test. The 400/200 ratio is 2.13, inside the normal 2.10–2.20 band, so the number is internally consistent. What the ratio cannot detect is both swims being submaximal together, and that now looks like what happened: on Oct 5 the warm-up 400 came in at 7:07.5 and the 5 × 200 that followed averaged 1:47.6/100 without fading. Treat 1:53 as a soft floor rather than a true threshold until Nov 9 re-measures it.</t>
         </is>
       </c>
     </row>
@@ -12550,7 +12550,7 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Now (Sep 21)</t>
+          <t>Sep 21 baseline</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -12572,29 +12572,29 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Good — 4 s/100 faster</t>
+          <t>Floor — an honest test, no fitness gained</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>6:58</t>
+          <t>7:00</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>3:20</t>
+          <t>3:18</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>1:49</t>
+          <t>1:51</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Strong — 6 s/100 faster</t>
+          <t>Good — the number to aim at</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -12604,427 +12604,449 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>3:18</t>
+          <t>3:16</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>1:47</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="35" t="inlineStr">
-        <is>
-          <t>Run the protocol identically — 400 first, 5 min full rest, then 200 — or the comparison means nothing. A sandbagged 200 inflates CSS and makes the block look better than it was, so both efforts have to be genuine.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="28" t="inlineStr">
+          <t>1:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>6:44</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>3:12</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>1:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>Two execution notes, both learned the hard way. First, warm up genuinely easy — 2:08–2:13/100, not the 1:45s of the last two sessions — because a 400 TT off a hard warm-up is just a second hard swim. Second, pace the 400 off the clock and not off feel: 1:42 for the first 100, 1:43s through the middle, empty the tank on the last 50. Then 5 min full rest before the 200. Run the protocol identically or the comparison means nothing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="28" t="inlineStr">
         <is>
           <t>Pace zones (recalculate off your measured CSS)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Zone</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Cue</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Easy / recovery</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>2:08–2:13</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>CSS + 15–20 s. Conversational. Warm-up, cool-down, and the technique swim.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Aerobic (Z2)</t>
+          <t>Easy / recovery</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>2:01–2:05</t>
+          <t>2:08–2:13</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>CSS + 8–12 s. What a long continuous swim should feel like. Nose-breathing calm.</t>
+          <t>CSS + 15–20 s. Conversational. Warm-up, cool-down, and the technique swim.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>CSS / threshold</t>
+          <t>Aerobic (Z2)</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>1:51–1:55</t>
+          <t>2:01–2:05</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Your tested 1:53, give or take 2 s. The engine of this block — comfortably hard, repeatable for 20–40 min of work.</t>
+          <t>CSS + 8–12 s. What a long continuous swim should feel like. Nose-breathing calm.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Fast (VO2)</t>
+          <t>CSS / threshold</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>1:45–1:48</t>
+          <t>1:51–1:55</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>CSS −5 to −8 s. 50s and short 100s, still with a clean catch and a long stroke.</t>
+          <t>Your tested 1:53, give or take 2 s. The engine of this block — comfortably hard, repeatable for 20–40 min of work.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
+          <t>Fast (VO2)</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>1:45–1:48</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>CSS −5 to −8 s. 50s and short 100s, still with a clean catch and a long stroke.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>1:35–1:40</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>25s and the last 50 of a set. 1:40 is your 200 TT pace — anything quicker is a genuine sprint, so use it sparingly.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="28" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="28" t="inlineStr">
         <is>
           <t>Send-offs</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>Set</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Send-off</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>Rest</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="7" t="inlineStr">
-        <is>
-          <t>100 aerobic</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>2:30</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>~27 s</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>100 threshold (CSS)</t>
+          <t>100 aerobic</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>2:15</t>
+          <t>2:30</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>~22 s</t>
+          <t>~27 s</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>100 fast</t>
+          <t>100 threshold (CSS)</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>2:30</t>
+          <t>2:15</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>~43 s</t>
+          <t>~22 s</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>50 aerobic</t>
+          <t>100 fast</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>1:15</t>
+          <t>2:30</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>~13 s</t>
+          <t>~43 s</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>50 threshold (CSS)</t>
+          <t>50 aerobic</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>1:05</t>
+          <t>1:15</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>~8 s</t>
+          <t>~13 s</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>50 fast</t>
+          <t>50 threshold (CSS)</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>1:15</t>
+          <t>1:05</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>~22 s</t>
+          <t>~8 s</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
+          <t>50 fast</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>1:15</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>~22 s</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
           <t>200 threshold (CSS)</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>4:25</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>~39 s</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="28" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="28" t="inlineStr">
         <is>
           <t>Drill progression</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>Focus</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="D38" s="3" t="inlineStr">
         <is>
           <t>Drills</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>Weeks 1–3</t>
-        </is>
-      </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>Body position + the send-off habit</t>
-        </is>
-      </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t>Get the new gear working and stop the sessions from being rest-dominated. Snorkel removes breathing as a variable so body and head position can actually be felt.</t>
-        </is>
-      </c>
-      <c r="D38" s="7" t="inlineStr">
-        <is>
-          <t>Snorkel + fins, 6 × 50: flutter kick on front, eyes down, hips high. · 6-1-6 with fins, 4 × 50 per side: six kicks on the side, one stroke, six on the other. · Catch-up, 4 × 50: patient lead arm, long body line, no crossover. · Fingertip drag, 4 × 50: relaxed recovery, high elbow, unhurried rotation. · Breathe-3 on easy 50s only — warm-up and cool-down, never inside a hard set. · Left-side ladder starts here: side kick (left) until stable, then side kick + breathe.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Weeks 4–7</t>
+          <t>Weeks 1–3</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Catch + symmetry</t>
+          <t>Body position + the send-off habit</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Build an earlier, higher-elbow catch and start balancing the stroke. Paddles arrive in Week 5 and stay capped.</t>
+          <t>Get the new gear working and stop the sessions from being rest-dominated. Snorkel removes breathing as a variable so body and head position can actually be felt.</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Front scull, 3 × 50 with snorkel: forearm vertical, pressure back not down. · Single-arm freestyle, 4 × 50 per side: the weak (left-breathing) side gets the extra 50. · Left-breathing single-arm, 4 × 50 with fins: right arm as a rail, breathe left every stroke. · Closed-fist, 4 × 50, then 50 normal — the contrast teaches the forearm to grip water. · 3/5/3 breathing pattern through warm-ups: three strokes, five strokes, three. · Small paddles + pull buoy, max 400 yd: hold the catch, stop if the shoulder complains. · Breaststroke timing, 4 × 50: pull, breathe, kick, glide — one thing at a time.</t>
+          <t>Snorkel + fins, 6 × 50: flutter kick on front, eyes down, hips high. · 6-1-6 with fins, 4 × 50 per side: six kicks on the side, one stroke, six on the other. · Catch-up, 4 × 50: patient lead arm, long body line, no crossover. · Fingertip drag, 4 × 50: relaxed recovery, high elbow, unhurried rotation. · Breathe-3 on easy 50s only — warm-up and cool-down, never inside a hard set. · Left-side ladder starts here: side kick (left) until stable, then side kick + breathe.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
+          <t>Weeks 4–7</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Catch + symmetry</t>
+        </is>
+      </c>
+      <c r="C40" s="7" t="inlineStr">
+        <is>
+          <t>Build an earlier, higher-elbow catch and start balancing the stroke. Paddles arrive in Week 5 and stay capped.</t>
+        </is>
+      </c>
+      <c r="D40" s="7" t="inlineStr">
+        <is>
+          <t>Front scull, 3 × 50 with snorkel: forearm vertical, pressure back not down. · Single-arm freestyle, 4 × 50 per side: the weak (left-breathing) side gets the extra 50. · Left-breathing single-arm, 4 × 50 with fins: right arm as a rail, breathe left every stroke. · Closed-fist, 4 × 50, then 50 normal — the contrast teaches the forearm to grip water. · 3/5/3 breathing pattern through warm-ups: three strokes, five strokes, three. · Small paddles + pull buoy, max 400 yd: hold the catch, stop if the shoulder complains. · Breaststroke timing, 4 × 50: pull, breathe, kick, glide — one thing at a time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
           <t>Weeks 8–15</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>Hold form under fatigue</t>
         </is>
       </c>
-      <c r="C40" s="7" t="inlineStr">
+      <c r="C41" s="7" t="inlineStr">
         <is>
           <t>Technique that survives a hard set is the only technique that counts. Stroke count and SWOLF become the feedback loop since there is no coach on deck.</t>
         </is>
       </c>
-      <c r="D40" s="7" t="inlineStr">
+      <c r="D41" s="7" t="inlineStr">
         <is>
           <t>Stroke-count ladder, 4 × 50: hold a fixed count per length, then drop it by one. · Descending 100s at a fixed stroke count — get faster without adding strokes. · Breathe-3 on easy 50s with rest, and only inside continuous swimming once the left breath survives those. · Sighting, 6 × 50: eyes just above the water every 6–8 strokes, ahead of open water next year. · Breaststroke 200 continuous — an honest second stroke, not a novelty. · Self-check every Monday: log the 100 that felt best and its stroke count.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="28" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="28" t="inlineStr">
         <is>
           <t>Before every swim</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>Checklist</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="7" t="inlineStr">
-        <is>
-          <t>Fins and center-mount snorkel in the bag from Week 1; small paddles bought before Week 5, which is when they enter.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>Know your CSS number and carry the send-off table on your phone.</t>
+          <t>Fins and center-mount snorkel in the bag from Week 1; small paddles bought before Week 5, which is when they enter.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>Every main set leaves on the clock — if you are resting until you feel ready, the set is wrong.</t>
+          <t>Know your CSS number and carry the send-off table on your phone.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>Stroke count per 25 yd logged on the best 100 of each Monday session.</t>
+          <t>Every main set leaves on the clock — if you are resting until you feel ready, the set is wrong.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>Left-side breathing competent — calm on easy 50s with rest by Week 7, inside continuous swimming by Week 10.</t>
+          <t>Stroke count per 25 yd logged on the best 100 of each Monday session.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>Breaststroke 200 continuous, relaxed, by Week 12.</t>
+          <t>Left-side breathing competent — calm on easy 50s with rest by Week 7, inside continuous swimming by Week 10.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>Breaststroke 200 continuous, relaxed, by Week 12.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
         <is>
           <t>Shoulder pain stays ≤ 2/10 — paddles are the first thing to drop if it does not.</t>
         </is>
@@ -13033,8 +13055,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Count the paddle pull inside the speed-50s swim totals
The Oct 21, Nov 11 and Nov 18 speed swims each prescribed a 400 paddle pull that was never counted in the session yardage, so the real swims ran 400 yd over the labeled total. The pull was also written as 'PADDLES:' / 'Paddles 400', which the app filed under Why / how instead of the session steps.

Totals stay as labeled; the pull now fits inside them and ramps in gradually: Oct 21 pull 200 + 20 x 50 (was 24), Nov 11 pull 200 + 5 rounds of 4 x 50 (was 6), Nov 18 pull 300 + 24 x 50 (was 30). Each pull line now starts with 'Pull' so it renders as a step between the drills and the main set.

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Abid — Fall 2026 Training Block.xlsx
+++ b/Abid — Fall 2026 Training Block.xlsx
@@ -3808,7 +3808,7 @@
       </c>
       <c r="F67" s="7" t="inlineStr">
         <is>
-          <t>Swim — speed 24 × 50 + first paddles</t>
+          <t>Swim — speed 20 × 50 + first paddles</t>
         </is>
       </c>
       <c r="G67" s="5" t="inlineStr">
@@ -3828,7 +3828,7 @@
       <c r="O67" s="13" t="n"/>
       <c r="P67" s="7" t="inlineStr">
         <is>
-          <t>Warm-up 300. Drill 400 as 8 × 50, each drill twice: closed-fist / catch-up / 6-1-6 / breaststroke timing. Fins throughout; snorkel off for 6-1-6 and breaststroke timing. PADDLES: 400 pull with small paddles and buoy, easy, holding the catch — stop immediately if the shoulder complains. Main: 24 × 50 on 1:05, alternating aerobic and fast. Then 4 × 50 breaststroke. Cool-down 200.</t>
+          <t>Warm-up 300. Drill 400 as 8 × 50, each drill twice: closed-fist / catch-up / 6-1-6 / breaststroke timing. Fins throughout; snorkel off for 6-1-6 and breaststroke timing. Pull 200 with small paddles and buoy, easy, holding the catch — first time on paddles, so 200 is plenty; stop immediately if the shoulder complains. Main: 20 × 50 on 1:05, alternating aerobic and fast. Then 4 × 50 breaststroke. Cool-down 200.</t>
         </is>
       </c>
     </row>
@@ -5764,7 +5764,7 @@
       </c>
       <c r="F107" s="7" t="inlineStr">
         <is>
-          <t>Swim — speed 6 × (4 × 50)</t>
+          <t>Swim — speed 5 × (4 × 50)</t>
         </is>
       </c>
       <c r="G107" s="5" t="inlineStr">
@@ -5784,7 +5784,7 @@
       <c r="O107" s="13" t="n"/>
       <c r="P107" s="7" t="inlineStr">
         <is>
-          <t>Warm-up 300. Drill 400 as 8 × 50, each drill twice: stroke-count ladder / front scull / 6-1-6 / closed-fist. Fins throughout; snorkel off for 6-1-6. Paddles 400 pull. Main: 6 rounds of 4 × 50 on 1:00, 45 s between rounds. Then 4 × 50 breaststroke. Cool-down 200. Tighter send-off than Week 5 — this is where density shows up.</t>
+          <t>Warm-up 300. Drill 400 as 8 × 50, each drill twice: stroke-count ladder / front scull / 6-1-6 / closed-fist. Fins throughout; snorkel off for 6-1-6. Pull 200 with small paddles and buoy, easy, holding the catch. Main: 5 rounds of 4 × 50 on 1:00, 45 s between rounds. Then 4 × 50 breaststroke. Cool-down 200. Tighter send-off than Week 5 — this is where density shows up.</t>
         </is>
       </c>
     </row>
@@ -6450,7 +6450,7 @@
       </c>
       <c r="F121" s="7" t="inlineStr">
         <is>
-          <t>Swim — speed 30 × 50</t>
+          <t>Swim — speed 24 × 50</t>
         </is>
       </c>
       <c r="G121" s="5" t="inlineStr">
@@ -6470,7 +6470,7 @@
       <c r="O121" s="13" t="n"/>
       <c r="P121" s="7" t="inlineStr">
         <is>
-          <t>Warm-up 300. Drill 400 as 8 × 50, each drill twice: 6-1-6 / closed-fist / sighting / breaststroke timing. Fins throughout; snorkel off for 6-1-6, sighting and breaststroke timing. Paddles 400. Main: 30 × 50 on 1:05, alternating aerobic and fast. Then 4 × 50 breaststroke. Cool-down 200. Long 50s set — the goal is that number 30 looks like number 1.</t>
+          <t>Warm-up 300. Drill 400 as 8 × 50, each drill twice: 6-1-6 / closed-fist / sighting / breaststroke timing. Fins throughout; snorkel off for 6-1-6, sighting and breaststroke timing. Pull 300 with small paddles and buoy, easy, holding the catch. Main: 24 × 50 on 1:05, alternating aerobic and fast. Then 4 × 50 breaststroke. Cool-down 200. Long 50s set — the goal is that number 24 looks like number 1.</t>
         </is>
       </c>
     </row>

</xml_diff>